<commit_message>
Support multiple privilege worksheets
</commit_message>
<xml_diff>
--- a/sample_data/privilegios.xlsx
+++ b/sample_data/privilegios.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diegotoscana/Library/CloudStorage/Dropbox/Diego's Dropbox/AnesthesiaCopilot/sample_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diegotoscana/Projects/AnesthesiaCopilot/sample_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34E31841-FB93-4947-8A9D-EEF1D91F9E23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96D78F53-7DED-3548-BC81-08505568BD9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="16460" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
-    <sheet name="Privilegios" sheetId="2" r:id="rId2"/>
+    <sheet name="Pediatricos" sheetId="3" r:id="rId2"/>
+    <sheet name="VTE Lopez" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -506,6 +507,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{499B7D99-3603-B143-9C10-80D1F1C70235}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
Add generic privilege service and pediatric validator
</commit_message>
<xml_diff>
--- a/sample_data/privilegios.xlsx
+++ b/sample_data/privilegios.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diegotoscana/Projects/AnesthesiaCopilot/sample_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96D78F53-7DED-3548-BC81-08505568BD9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{862B1D2F-2C19-F04D-A0CF-A8ACC3510554}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="16460" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="16460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
-    <sheet name="Pediatricos" sheetId="3" r:id="rId2"/>
+    <sheet name="Pediátricos" sheetId="3" r:id="rId2"/>
     <sheet name="VTE Lopez" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
   <si>
     <t>Privilegios - VTE López</t>
   </si>
@@ -85,6 +85,27 @@
   </si>
   <si>
     <t>Costales</t>
+  </si>
+  <si>
+    <t>Donis</t>
+  </si>
+  <si>
+    <t>Ronconi</t>
+  </si>
+  <si>
+    <t>Lafuente</t>
+  </si>
+  <si>
+    <t>Megadiaz</t>
+  </si>
+  <si>
+    <t>Torres</t>
+  </si>
+  <si>
+    <t>Resio</t>
+  </si>
+  <si>
+    <t>Sanchez Crocci</t>
   </si>
 </sst>
 </file>
@@ -508,9 +529,53 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{499B7D99-3603-B143-9C10-80D1F1C70235}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="40" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add surgeon incompatibility validator
</commit_message>
<xml_diff>
--- a/sample_data/privilegios.xlsx
+++ b/sample_data/privilegios.xlsx
@@ -8,21 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diegotoscana/Projects/AnesthesiaCopilot/sample_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{862B1D2F-2C19-F04D-A0CF-A8ACC3510554}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDF720BA-68F8-3A46-A60B-C63A5D432974}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="16460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="560" yWindow="1820" windowWidth="28800" windowHeight="16460" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
     <sheet name="Pediátricos" sheetId="3" r:id="rId2"/>
-    <sheet name="VTE Lopez" sheetId="2" r:id="rId3"/>
+    <sheet name="Incompatibilidades" sheetId="4" r:id="rId3"/>
+    <sheet name="VTE Lopez" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="36">
   <si>
     <t>Privilegios - VTE López</t>
   </si>
@@ -106,13 +107,37 @@
   </si>
   <si>
     <t>Sanchez Crocci</t>
+  </si>
+  <si>
+    <t>Cirujano</t>
+  </si>
+  <si>
+    <t>Gómez</t>
+  </si>
+  <si>
+    <t>Loncharich</t>
+  </si>
+  <si>
+    <t>Lloyd</t>
+  </si>
+  <si>
+    <t>Hwang</t>
+  </si>
+  <si>
+    <t>Barbieri</t>
+  </si>
+  <si>
+    <t>Cameron</t>
+  </si>
+  <si>
+    <t>MAYA ANTONIO GUSTAVO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -131,6 +156,14 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -163,11 +196,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -581,6 +615,68 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{353CB2CE-9CBC-F646-A85A-3BFDF416AFF6}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>

</xml_diff>